<commit_message>
data backup + FII/DII refresh (2026-09-21)
</commit_message>
<xml_diff>
--- a/fii-dii/FII_DII_History.xlsx
+++ b/fii-dii/FII_DII_History.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I612"/>
+  <dimension ref="A1:I618"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -29088,6 +29088,288 @@
         </is>
       </c>
       <c r="I612" t="inlineStr">
+        <is>
+          <t>provisional</t>
+        </is>
+      </c>
+    </row>
+    <row r="613">
+      <c r="A613" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B613" t="inlineStr">
+        <is>
+          <t>11882.95</t>
+        </is>
+      </c>
+      <c r="C613" t="inlineStr">
+        <is>
+          <t>12321.19</t>
+        </is>
+      </c>
+      <c r="D613" t="inlineStr">
+        <is>
+          <t>-438.24</t>
+        </is>
+      </c>
+      <c r="E613" t="inlineStr">
+        <is>
+          <t>13326.33</t>
+        </is>
+      </c>
+      <c r="F613" t="inlineStr">
+        <is>
+          <t>12300.48</t>
+        </is>
+      </c>
+      <c r="G613" t="inlineStr">
+        <is>
+          <t>1025.85</t>
+        </is>
+      </c>
+      <c r="H613" t="inlineStr">
+        <is>
+          <t>Groww</t>
+        </is>
+      </c>
+      <c r="I613" t="inlineStr">
+        <is>
+          <t>provisional</t>
+        </is>
+      </c>
+    </row>
+    <row r="614">
+      <c r="A614" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="B614" t="inlineStr">
+        <is>
+          <t>12616.89</t>
+        </is>
+      </c>
+      <c r="C614" t="inlineStr">
+        <is>
+          <t>13547.79</t>
+        </is>
+      </c>
+      <c r="D614" t="inlineStr">
+        <is>
+          <t>-930.9</t>
+        </is>
+      </c>
+      <c r="E614" t="inlineStr">
+        <is>
+          <t>15109.58</t>
+        </is>
+      </c>
+      <c r="F614" t="inlineStr">
+        <is>
+          <t>13141.41</t>
+        </is>
+      </c>
+      <c r="G614" t="inlineStr">
+        <is>
+          <t>1968.17</t>
+        </is>
+      </c>
+      <c r="H614" t="inlineStr">
+        <is>
+          <t>Groww</t>
+        </is>
+      </c>
+      <c r="I614" t="inlineStr">
+        <is>
+          <t>provisional</t>
+        </is>
+      </c>
+    </row>
+    <row r="615">
+      <c r="A615" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="B615" t="inlineStr">
+        <is>
+          <t>13194.76</t>
+        </is>
+      </c>
+      <c r="C615" t="inlineStr">
+        <is>
+          <t>16172.62</t>
+        </is>
+      </c>
+      <c r="D615" t="inlineStr">
+        <is>
+          <t>-2977.86</t>
+        </is>
+      </c>
+      <c r="E615" t="inlineStr">
+        <is>
+          <t>15221.98</t>
+        </is>
+      </c>
+      <c r="F615" t="inlineStr">
+        <is>
+          <t>12535.93</t>
+        </is>
+      </c>
+      <c r="G615" t="inlineStr">
+        <is>
+          <t>2686.05</t>
+        </is>
+      </c>
+      <c r="H615" t="inlineStr">
+        <is>
+          <t>Groww</t>
+        </is>
+      </c>
+      <c r="I615" t="inlineStr">
+        <is>
+          <t>provisional</t>
+        </is>
+      </c>
+    </row>
+    <row r="616">
+      <c r="A616" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B616" t="inlineStr">
+        <is>
+          <t>12959.04</t>
+        </is>
+      </c>
+      <c r="C616" t="inlineStr">
+        <is>
+          <t>14991.65</t>
+        </is>
+      </c>
+      <c r="D616" t="inlineStr">
+        <is>
+          <t>-2032.61</t>
+        </is>
+      </c>
+      <c r="E616" t="inlineStr">
+        <is>
+          <t>15279.59</t>
+        </is>
+      </c>
+      <c r="F616" t="inlineStr">
+        <is>
+          <t>11371.36</t>
+        </is>
+      </c>
+      <c r="G616" t="inlineStr">
+        <is>
+          <t>3908.23</t>
+        </is>
+      </c>
+      <c r="H616" t="inlineStr">
+        <is>
+          <t>Groww</t>
+        </is>
+      </c>
+      <c r="I616" t="inlineStr">
+        <is>
+          <t>provisional</t>
+        </is>
+      </c>
+    </row>
+    <row r="617">
+      <c r="A617" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="B617" t="inlineStr">
+        <is>
+          <t>8761.71</t>
+        </is>
+      </c>
+      <c r="C617" t="inlineStr">
+        <is>
+          <t>11970.47</t>
+        </is>
+      </c>
+      <c r="D617" t="inlineStr">
+        <is>
+          <t>-3208.76</t>
+        </is>
+      </c>
+      <c r="E617" t="inlineStr">
+        <is>
+          <t>14105.01</t>
+        </is>
+      </c>
+      <c r="F617" t="inlineStr">
+        <is>
+          <t>10487.26</t>
+        </is>
+      </c>
+      <c r="G617" t="inlineStr">
+        <is>
+          <t>3617.75</t>
+        </is>
+      </c>
+      <c r="H617" t="inlineStr">
+        <is>
+          <t>Groww</t>
+        </is>
+      </c>
+      <c r="I617" t="inlineStr">
+        <is>
+          <t>provisional</t>
+        </is>
+      </c>
+    </row>
+    <row r="618">
+      <c r="A618" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="B618" t="inlineStr">
+        <is>
+          <t>38461.63</t>
+        </is>
+      </c>
+      <c r="C618" t="inlineStr">
+        <is>
+          <t>37862.09</t>
+        </is>
+      </c>
+      <c r="D618" t="inlineStr">
+        <is>
+          <t>599.54</t>
+        </is>
+      </c>
+      <c r="E618" t="inlineStr">
+        <is>
+          <t>17310.04</t>
+        </is>
+      </c>
+      <c r="F618" t="inlineStr">
+        <is>
+          <t>16290.35</t>
+        </is>
+      </c>
+      <c r="G618" t="inlineStr">
+        <is>
+          <t>1019.69</t>
+        </is>
+      </c>
+      <c r="H618" t="inlineStr">
+        <is>
+          <t>Site-edge</t>
+        </is>
+      </c>
+      <c r="I618" t="inlineStr">
         <is>
           <t>provisional</t>
         </is>

</xml_diff>

<commit_message>
data backup + FII/DII refresh (2026-09-22)
</commit_message>
<xml_diff>
--- a/fii-dii/FII_DII_History.xlsx
+++ b/fii-dii/FII_DII_History.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I618"/>
+  <dimension ref="A1:I619"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -29370,6 +29370,53 @@
         </is>
       </c>
       <c r="I618" t="inlineStr">
+        <is>
+          <t>provisional</t>
+        </is>
+      </c>
+    </row>
+    <row r="619">
+      <c r="A619" t="inlineStr">
+        <is>
+          <t>2026-09-21</t>
+        </is>
+      </c>
+      <c r="B619" t="inlineStr">
+        <is>
+          <t>10637.17</t>
+        </is>
+      </c>
+      <c r="C619" t="inlineStr">
+        <is>
+          <t>11213.37</t>
+        </is>
+      </c>
+      <c r="D619" t="inlineStr">
+        <is>
+          <t>-576.2</t>
+        </is>
+      </c>
+      <c r="E619" t="inlineStr">
+        <is>
+          <t>14098.64</t>
+        </is>
+      </c>
+      <c r="F619" t="inlineStr">
+        <is>
+          <t>11301.37</t>
+        </is>
+      </c>
+      <c r="G619" t="inlineStr">
+        <is>
+          <t>2797.27</t>
+        </is>
+      </c>
+      <c r="H619" t="inlineStr">
+        <is>
+          <t>Site-edge</t>
+        </is>
+      </c>
+      <c r="I619" t="inlineStr">
         <is>
           <t>provisional</t>
         </is>

</xml_diff>

<commit_message>
data backup + FII/DII refresh (2026-09-23)
</commit_message>
<xml_diff>
--- a/fii-dii/FII_DII_History.xlsx
+++ b/fii-dii/FII_DII_History.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I619"/>
+  <dimension ref="A1:I620"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -29417,6 +29417,53 @@
         </is>
       </c>
       <c r="I619" t="inlineStr">
+        <is>
+          <t>provisional</t>
+        </is>
+      </c>
+    </row>
+    <row r="620">
+      <c r="A620" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="B620" t="inlineStr">
+        <is>
+          <t>9845.81</t>
+        </is>
+      </c>
+      <c r="C620" t="inlineStr">
+        <is>
+          <t>13655.8</t>
+        </is>
+      </c>
+      <c r="D620" t="inlineStr">
+        <is>
+          <t>-3809.99</t>
+        </is>
+      </c>
+      <c r="E620" t="inlineStr">
+        <is>
+          <t>14599.72</t>
+        </is>
+      </c>
+      <c r="F620" t="inlineStr">
+        <is>
+          <t>10479.65</t>
+        </is>
+      </c>
+      <c r="G620" t="inlineStr">
+        <is>
+          <t>4120.07</t>
+        </is>
+      </c>
+      <c r="H620" t="inlineStr">
+        <is>
+          <t>Site-edge</t>
+        </is>
+      </c>
+      <c r="I620" t="inlineStr">
         <is>
           <t>provisional</t>
         </is>

</xml_diff>

<commit_message>
data backup + FII/DII refresh (2026-09-24)
</commit_message>
<xml_diff>
--- a/fii-dii/FII_DII_History.xlsx
+++ b/fii-dii/FII_DII_History.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I620"/>
+  <dimension ref="A1:I621"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -29464,6 +29464,53 @@
         </is>
       </c>
       <c r="I620" t="inlineStr">
+        <is>
+          <t>provisional</t>
+        </is>
+      </c>
+    </row>
+    <row r="621">
+      <c r="A621" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="B621" t="inlineStr">
+        <is>
+          <t>13580.4</t>
+        </is>
+      </c>
+      <c r="C621" t="inlineStr">
+        <is>
+          <t>11962.95</t>
+        </is>
+      </c>
+      <c r="D621" t="inlineStr">
+        <is>
+          <t>1617.45</t>
+        </is>
+      </c>
+      <c r="E621" t="inlineStr">
+        <is>
+          <t>14404.9</t>
+        </is>
+      </c>
+      <c r="F621" t="inlineStr">
+        <is>
+          <t>12063.44</t>
+        </is>
+      </c>
+      <c r="G621" t="inlineStr">
+        <is>
+          <t>2341.46</t>
+        </is>
+      </c>
+      <c r="H621" t="inlineStr">
+        <is>
+          <t>Site-edge</t>
+        </is>
+      </c>
+      <c r="I621" t="inlineStr">
         <is>
           <t>provisional</t>
         </is>

</xml_diff>

<commit_message>
data backup + FII/DII refresh (2026-09-29)
</commit_message>
<xml_diff>
--- a/fii-dii/FII_DII_History.xlsx
+++ b/fii-dii/FII_DII_History.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I621"/>
+  <dimension ref="A1:I624"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -29511,6 +29511,147 @@
         </is>
       </c>
       <c r="I621" t="inlineStr">
+        <is>
+          <t>provisional</t>
+        </is>
+      </c>
+    </row>
+    <row r="622">
+      <c r="A622" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B622" t="inlineStr">
+        <is>
+          <t>13111.22</t>
+        </is>
+      </c>
+      <c r="C622" t="inlineStr">
+        <is>
+          <t>18138.58</t>
+        </is>
+      </c>
+      <c r="D622" t="inlineStr">
+        <is>
+          <t>-5027.36</t>
+        </is>
+      </c>
+      <c r="E622" t="inlineStr">
+        <is>
+          <t>18196.9</t>
+        </is>
+      </c>
+      <c r="F622" t="inlineStr">
+        <is>
+          <t>13895.72</t>
+        </is>
+      </c>
+      <c r="G622" t="inlineStr">
+        <is>
+          <t>4301.18</t>
+        </is>
+      </c>
+      <c r="H622" t="inlineStr">
+        <is>
+          <t>Groww</t>
+        </is>
+      </c>
+      <c r="I622" t="inlineStr">
+        <is>
+          <t>provisional</t>
+        </is>
+      </c>
+    </row>
+    <row r="623">
+      <c r="A623" t="inlineStr">
+        <is>
+          <t>2026-09-25</t>
+        </is>
+      </c>
+      <c r="B623" t="inlineStr">
+        <is>
+          <t>12327.36</t>
+        </is>
+      </c>
+      <c r="C623" t="inlineStr">
+        <is>
+          <t>16021.29</t>
+        </is>
+      </c>
+      <c r="D623" t="inlineStr">
+        <is>
+          <t>-3693.93</t>
+        </is>
+      </c>
+      <c r="E623" t="inlineStr">
+        <is>
+          <t>14035.77</t>
+        </is>
+      </c>
+      <c r="F623" t="inlineStr">
+        <is>
+          <t>11197.6</t>
+        </is>
+      </c>
+      <c r="G623" t="inlineStr">
+        <is>
+          <t>2838.17</t>
+        </is>
+      </c>
+      <c r="H623" t="inlineStr">
+        <is>
+          <t>Groww</t>
+        </is>
+      </c>
+      <c r="I623" t="inlineStr">
+        <is>
+          <t>provisional</t>
+        </is>
+      </c>
+    </row>
+    <row r="624">
+      <c r="A624" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="B624" t="inlineStr">
+        <is>
+          <t>9047.56</t>
+        </is>
+      </c>
+      <c r="C624" t="inlineStr">
+        <is>
+          <t>14400.78</t>
+        </is>
+      </c>
+      <c r="D624" t="inlineStr">
+        <is>
+          <t>-5353.22</t>
+        </is>
+      </c>
+      <c r="E624" t="inlineStr">
+        <is>
+          <t>15918.32</t>
+        </is>
+      </c>
+      <c r="F624" t="inlineStr">
+        <is>
+          <t>10729.3</t>
+        </is>
+      </c>
+      <c r="G624" t="inlineStr">
+        <is>
+          <t>5189.02</t>
+        </is>
+      </c>
+      <c r="H624" t="inlineStr">
+        <is>
+          <t>Site-edge</t>
+        </is>
+      </c>
+      <c r="I624" t="inlineStr">
         <is>
           <t>provisional</t>
         </is>

</xml_diff>